<commit_message>
Fix 26-07-14_4: village win should have included Mistici (Veggente/Giorgio was missing from win_ruoli)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -5456,12 +5456,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Villaggio</t>
+          <t>Villaggio, Mistici</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bocca di Rosa, Borgomastro, Fanatico, Guardia, Peccatore</t>
+          <t>Bocca di Rosa, Borgomastro, Fanatico, Guardia, Peccatore, Veggente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game 26-06-17_2: Villaggio/Mistici win (Strega, Veggente, Monaco, Mercante, Bocca di Rosa)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -2909,7 +2909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V35"/>
+  <dimension ref="A1:W35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3029,6 +3029,11 @@
           <t>26-07-14_4</t>
         </is>
       </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>26-06-17_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3295,6 +3300,11 @@
           <t>Peccatore</t>
         </is>
       </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3369,6 +3379,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>Mercante</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3436,6 +3451,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Bocca di Rosa</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3513,6 +3533,11 @@
           <t>Guardia Corrotta</t>
         </is>
       </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3627,6 +3652,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3709,6 +3739,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Pazzo</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3858,6 +3893,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4208,6 +4248,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4303,6 +4348,11 @@
       <c r="V24" t="inlineStr">
         <is>
           <t>MASTER</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
         </is>
       </c>
     </row>
@@ -4575,7 +4625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -4831,6 +4881,18 @@
       <c r="B21" t="inlineStr">
         <is>
           <t>2 lune NO Giullare, sì Fanatico, sì Sensitiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>26-06-17_2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare</t>
         </is>
       </c>
     </row>
@@ -4846,7 +4908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5090,6 +5152,18 @@
       <c r="B20" t="inlineStr">
         <is>
           <t>Fanatico di Bocca di Rosa</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>26-06-17_2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Monaco no Spia, Prete, Medium, Mago</t>
         </is>
       </c>
     </row>
@@ -5105,7 +5179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5462,6 +5536,23 @@
       <c r="C21" t="inlineStr">
         <is>
           <t>Bocca di Rosa, Borgomastro, Fanatico, Guardia, Peccatore, Veggente</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>26-06-17_2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Veggente, Strega, Monaco, Bocca di Rosa, Mercante</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Normalize Ruoli Possibili text across all games: no commas, NO/SÌ always uppercase, faida lupi -> faida, Giullare first after NO then alphabetical, SÌ list purely alphabetical, merge duplicate SÌ clauses
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -4652,7 +4652,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, Strega</t>
+          <t>2 lune NO Giullare Strega</t>
         </is>
       </c>
     </row>
@@ -4724,7 +4724,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, Strega</t>
+          <t>2 lune NO Giullare Strega</t>
         </is>
       </c>
     </row>
@@ -4748,7 +4748,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, Vampiri</t>
+          <t>2 lune NO Giullare Vampiri</t>
         </is>
       </c>
     </row>
@@ -4784,7 +4784,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, Vampiri SÌ Fanatico, Faida</t>
+          <t>2 lune NO Giullare Vampiri SÌ Faida Fanatico</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4796,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, Vampiri</t>
+          <t>2 lune NO Giullare Vampiri</t>
         </is>
       </c>
     </row>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, Vampiri</t>
+          <t>2 lune NO Giullare Vampiri</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4832,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare SÌ Lupo Reietto, Lupo Solitario</t>
+          <t>2 lune NO Giullare SÌ Lupo Reietto Lupo Solitario</t>
         </is>
       </c>
     </row>
@@ -4844,7 +4844,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, amanti, sì faida lupi, megera, inquisitore</t>
+          <t>2 lune NO Giullare amanti SÌ faida inquisitore megera</t>
         </is>
       </c>
     </row>
@@ -4868,7 +4868,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, sì Fanatico, sì Sensitiva</t>
+          <t>2 lune NO Giullare SÌ Fanatico Sensitiva</t>
         </is>
       </c>
     </row>
@@ -4880,7 +4880,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare, sì Fanatico, sì Sensitiva</t>
+          <t>2 lune NO Giullare SÌ Fanatico Sensitiva</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix game dates: rename 26-07-14_3/_4 to 26-07-16_1/_2 (were actually played on the 16th, not the 14th)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3021,12 +3021,12 @@
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>26-07-14_3</t>
+          <t>26-07-16_1</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>26-07-14_4</t>
+          <t>26-07-16_2</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
@@ -4863,7 +4863,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>26-07-14_3</t>
+          <t>26-07-16_1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4875,7 +4875,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>26-07-14_4</t>
+          <t>26-07-16_2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5134,7 +5134,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>26-07-14_3</t>
+          <t>26-07-16_1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5146,7 +5146,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>26-07-14_4</t>
+          <t>26-07-16_2</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5508,7 +5508,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>26-07-14_3</t>
+          <t>26-07-16_1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5525,7 +5525,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>26-07-14_4</t>
+          <t>26-07-16_2</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5846,7 +5846,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>26-07-14_3</t>
+          <t>26-07-16_1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -5863,7 +5863,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>26-07-14_4</t>
+          <t>26-07-16_2</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">

</xml_diff>

<commit_message>
Add fan-made roles Capobranco Maledetto and Giullare Modificato; add game 26-07-23_1: Negromante win (Davide only)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -900,7 +900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="14.5546875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2894,6 +2894,70 @@
       <c r="G54" t="inlineStr">
         <is>
           <t>1 luna</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Ombra</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Fanmade</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Giullare Modificato</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Giullare</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Non Ombra</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Fanmade</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W35"/>
+  <dimension ref="A1:X35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3034,6 +3098,11 @@
           <t>26-06-17_2</t>
         </is>
       </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>26-07-23_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3136,6 +3205,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3188,6 +3262,11 @@
           <t>Cacciatore di Vampiri</t>
         </is>
       </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3305,6 +3384,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3456,6 +3540,11 @@
           <t>Bocca di Rosa</t>
         </is>
       </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>Giullare Modificato</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3657,6 +3746,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>Altra Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3781,6 +3875,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3898,6 +3997,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4174,6 +4278,11 @@
           <t>Mercante</t>
         </is>
       </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4355,6 +4464,11 @@
           <t>Vampiro</t>
         </is>
       </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4382,6 +4496,11 @@
           <t>Borgomastro</t>
         </is>
       </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>Negromante</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4424,6 +4543,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4476,6 +4600,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4610,6 +4739,11 @@
       <c r="V35" t="inlineStr">
         <is>
           <t>Bocca di Rosa</t>
+        </is>
+      </c>
+      <c r="X35" t="inlineStr">
+        <is>
+          <t>Capogilda</t>
         </is>
       </c>
     </row>
@@ -4625,7 +4759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -4893,6 +5027,18 @@
       <c r="B22" t="inlineStr">
         <is>
           <t>2 lune NO Giullare</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>26-07-23_1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Giullare Modificato Negromante</t>
         </is>
       </c>
     </row>
@@ -4908,7 +5054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5164,6 +5310,18 @@
       <c r="B21" t="inlineStr">
         <is>
           <t>Monaco no Spia, Prete, Medium, Mago</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>26-07-23_1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Monaco no Criminali tranne Capogilda; Maledetti Tullio e Filippo</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5553,6 +5711,23 @@
       <c r="C22" t="inlineStr">
         <is>
           <t>Veggente, Strega, Monaco, Bocca di Rosa, Mercante</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>26-07-23_1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Negromante</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Negromante</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5877,6 +6052,23 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>26-07-23_1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Ilaria</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Criminali</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-07-23_2: Capobranco/Fanatico win (Capobranco Maledetto, Lupo del Branco, Fanatico=Capobranco Maledetto)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -2973,7 +2973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X35"/>
+  <dimension ref="A1:Y35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3103,6 +3103,11 @@
           <t>26-07-23_1</t>
         </is>
       </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>26-07-23_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3210,6 +3215,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3389,6 +3399,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3751,6 +3766,11 @@
           <t>Altra Guardia</t>
         </is>
       </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3880,6 +3900,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4002,6 +4027,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4469,6 +4499,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4501,6 +4536,11 @@
           <t>Negromante</t>
         </is>
       </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4548,6 +4588,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4605,6 +4650,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="Y27" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4744,6 +4794,11 @@
       <c r="X35" t="inlineStr">
         <is>
           <t>Capogilda</t>
+        </is>
+      </c>
+      <c r="Y35" t="inlineStr">
+        <is>
+          <t>Veggente</t>
         </is>
       </c>
     </row>
@@ -4759,7 +4814,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5039,6 +5094,18 @@
       <c r="B23" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Giullare Modificato Negromante</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>26-07-23_2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare</t>
         </is>
       </c>
     </row>
@@ -5054,7 +5121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5322,6 +5389,18 @@
       <c r="B22" t="inlineStr">
         <is>
           <t>Monaco no Criminali tranne Capogilda; Maledetti Tullio e Filippo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>26-07-23_2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Angelo di Veggente, Fanatico di Capobranco Maledetto</t>
         </is>
       </c>
     </row>
@@ -5337,7 +5416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5728,6 +5807,23 @@
       <c r="C23" t="inlineStr">
         <is>
           <t>Negromante</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>26-07-23_2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Capobranco, Fanatico</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto, Fanatico, Lupo del Branco</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6069,6 +6165,23 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>26-07-23_2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>L'improbabile</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
26-07-23_1: add Medium gildato note, override Massimo's final condition to Criminali
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -5388,7 +5388,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Monaco no Criminali tranne Capogilda; Maledetti Tullio e Filippo</t>
+          <t>Monaco no Criminali tranne Capogilda; Maledetti Tullio e Filippo; Medium gildato</t>
         </is>
       </c>
     </row>
@@ -5839,7 +5839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6182,6 +6182,23 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>26-07-23_1</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Massimo</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Criminali</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add player Elena and game 26-07-30_1: Villaggio/Mistici win, Inquisitore=Romeo (Giulietta's target)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -881,6 +881,18 @@
       <c r="B35" t="inlineStr">
         <is>
           <t>Simone</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Elena</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Elena</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y35"/>
+  <dimension ref="A1:Z36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3108,6 +3120,11 @@
           <t>26-07-23_2</t>
         </is>
       </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>26-07-30_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3220,6 +3237,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Mercante</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3277,6 +3299,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3404,6 +3431,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3560,6 +3592,11 @@
           <t>Giullare Modificato</t>
         </is>
       </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3642,6 +3679,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>Giulietta</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3689,6 +3731,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3771,6 +3818,11 @@
           <t>Prete</t>
         </is>
       </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4032,6 +4084,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4104,6 +4161,11 @@
           <t>Oste</t>
         </is>
       </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Inquisitore</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4224,6 +4286,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4313,6 +4380,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4365,6 +4437,11 @@
           <t>Angelo</t>
         </is>
       </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Ladra</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4504,6 +4581,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4799,6 +4881,28 @@
       <c r="Y35" t="inlineStr">
         <is>
           <t>Veggente</t>
+        </is>
+      </c>
+      <c r="Z35" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Elena</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Elena</t>
+        </is>
+      </c>
+      <c r="Z36" t="inlineStr">
+        <is>
+          <t>Megera</t>
         </is>
       </c>
     </row>
@@ -4814,7 +4918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5104,6 +5208,18 @@
         </is>
       </c>
       <c r="B24" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>26-07-30_1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
         <is>
           <t>2 lune NO Giullare</t>
         </is>
@@ -5121,7 +5237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5401,6 +5517,18 @@
       <c r="B23" t="inlineStr">
         <is>
           <t>Angelo di Veggente, Fanatico di Capobranco Maledetto</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>26-07-30_1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Monaco no Ghoul, Traditore, Spia; Giulietta di Inquisitore</t>
         </is>
       </c>
     </row>
@@ -5416,7 +5544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5824,6 +5952,23 @@
       <c r="C24" t="inlineStr">
         <is>
           <t>Capobranco Maledetto, Fanatico, Lupo del Branco</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>26-07-30_1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Monaco, Eremita, Veggente, Guardia, Prete, Mercante, Cacciatore di Vampiri</t>
         </is>
       </c>
     </row>
@@ -5839,7 +5984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6199,6 +6344,23 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>26-07-30_1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Lu'</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Romeo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-07-30_2: Villaggio/Mistici win, Giovane Lupo=Romeo (Giulietta's target)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -2985,7 +2985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z36"/>
+  <dimension ref="A1:AA36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3125,6 +3125,11 @@
           <t>26-07-30_1</t>
         </is>
       </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>26-07-30_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3242,6 +3247,11 @@
           <t>Mercante</t>
         </is>
       </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3436,6 +3446,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3597,6 +3612,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Altra Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3684,6 +3704,11 @@
           <t>Giulietta</t>
         </is>
       </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3823,6 +3848,11 @@
           <t>Vampiro</t>
         </is>
       </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>Giulietta</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4089,6 +4119,11 @@
           <t>Prete</t>
         </is>
       </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4166,6 +4201,11 @@
           <t>Inquisitore</t>
         </is>
       </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4291,6 +4331,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>Borgomastro</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4584,6 +4629,11 @@
       <c r="Z24" t="inlineStr">
         <is>
           <t>Veggente</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5220,6 +5270,18 @@
         </is>
       </c>
       <c r="B25" t="inlineStr">
+        <is>
+          <t>2 lune NO Giullare</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>26-07-30_2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>2 lune NO Giullare</t>
         </is>
@@ -5237,7 +5299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5529,6 +5591,18 @@
       <c r="B24" t="inlineStr">
         <is>
           <t>Monaco no Ghoul, Traditore, Spia; Giulietta di Inquisitore</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>26-07-30_2</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Giulietta di Giovane Lupo</t>
         </is>
       </c>
     </row>
@@ -5544,7 +5618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5969,6 +6043,23 @@
       <c r="C25" t="inlineStr">
         <is>
           <t>Monaco, Eremita, Veggente, Guardia, Prete, Mercante, Cacciatore di Vampiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>26-07-30_2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Altra Guardia, Borgomastro, Eremita, Guardia, Veggente</t>
         </is>
       </c>
     </row>
@@ -5984,7 +6075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6361,6 +6452,23 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>26-07-30_2</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>La Regina</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Romeo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix 26-07-30_2: Luca was Giullare Modificato not Eremita (didn't win, removed from win_ruoli); correct Ruoli Possibili for both 26-07-30_1 and _2
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -4203,7 +4203,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>Eremita</t>
+          <t>Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare</t>
+          <t>2 lune NO Giullare SÌ Inquisizione Megera</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5283,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2 lune NO Giullare</t>
+          <t>2 lune SÌ Capobranco Maledetto Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6059,7 +6059,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Altra Guardia, Borgomastro, Eremita, Guardia, Veggente</t>
+          <t>Altra Guardia, Borgomastro, Guardia, Veggente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add players Andrea and GiorgioC; add game 26-08-21_1: Villaggio/Mistici win, Fanatico=Guardia's Villaggio
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B36"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -893,6 +893,30 @@
       <c r="B36" t="inlineStr">
         <is>
           <t>Elena</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Andrea</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Andrea</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>GiorgioC</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>GiorgioC</t>
         </is>
       </c>
     </row>
@@ -2985,7 +3009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA36"/>
+  <dimension ref="A1:AB38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3130,6 +3154,11 @@
           <t>26-07-30_2</t>
         </is>
       </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>26-08-21_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3617,6 +3646,11 @@
           <t>Altra Guardia</t>
         </is>
       </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Mago</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3709,6 +3743,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3853,6 +3892,11 @@
           <t>Giulietta</t>
         </is>
       </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>Assassino</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3940,6 +3984,11 @@
           <t>Pazzo</t>
         </is>
       </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4124,6 +4173,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4206,6 +4260,11 @@
           <t>Giullare Modificato</t>
         </is>
       </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4255,6 +4314,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>Azzeccagarbugli</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4430,6 +4494,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4725,6 +4794,11 @@
           <t>Eremita</t>
         </is>
       </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4953,6 +5027,40 @@
       <c r="Z36" t="inlineStr">
         <is>
           <t>Megera</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Andrea</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Andrea</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>Giullare</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>GiorgioC</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>GiorgioC</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
         </is>
       </c>
     </row>
@@ -4968,7 +5076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5284,6 +5392,18 @@
       <c r="B26" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26-08-21_1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5603,6 +5723,18 @@
       <c r="B25" t="inlineStr">
         <is>
           <t>Giulietta di Giovane Lupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>26-08-21_1</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Monaco no Contadino, Spia, Capogilda; Fanatico della Guardia</t>
         </is>
       </c>
     </row>
@@ -5618,7 +5750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6060,6 +6192,23 @@
       <c r="C26" t="inlineStr">
         <is>
           <t>Altra Guardia, Borgomastro, Guardia, Veggente</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26-08-21_1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Mago, Guardia, Azzeccagarbugli, Fanatico, Monaco, Veggente</t>
         </is>
       </c>
     </row>
@@ -6075,7 +6224,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6469,6 +6618,23 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>26-08-21_1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Giuseppe</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Villaggio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix 26-08-21_1: GiorgioC was actually Giorgio (ZicNick), not a new player; remove erroneous GiorgioC entry. Add player Alessio; add games 26-08-05_1 (Villaggio/Giullare/Mistici win, Margherita vampirizzata) and 26-08-11_1 (Villaggio/Mistici win)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -911,12 +911,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GiorgioC</t>
+          <t>Alessio</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GiorgioC</t>
+          <t>Alessio</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB38"/>
+  <dimension ref="A1:AD38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3159,6 +3159,16 @@
           <t>26-08-21_1</t>
         </is>
       </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>26-08-05_1</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>26-08-11_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3281,6 +3291,16 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>Guaritore</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3480,6 +3500,11 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Oratore</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3517,6 +3542,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3651,6 +3681,11 @@
           <t>Mago</t>
         </is>
       </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Bardo</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3800,6 +3835,11 @@
           <t>Eremita</t>
         </is>
       </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Giullare</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -3989,6 +4029,16 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4178,6 +4228,16 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>Mercante</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4265,6 +4325,16 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4432,6 +4502,16 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AC20" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Mercante</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4499,6 +4579,16 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4705,6 +4795,16 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>Cacciatore di Vampiri</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4799,6 +4899,11 @@
           <t>Fanatico</t>
         </is>
       </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>Contadino</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4861,6 +4966,16 @@
           <t>Angelo</t>
         </is>
       </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5050,17 +5165,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>GiorgioC</t>
+          <t>Alessio</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>GiorgioC</t>
-        </is>
-      </c>
-      <c r="AB38" t="inlineStr">
-        <is>
-          <t>Capobranco Maledetto</t>
+          <t>Alessio</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>Pazzo</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5402,6 +5517,30 @@
         </is>
       </c>
       <c r="B27" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>26-08-05_1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>26-08-11_1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
         </is>
@@ -5419,7 +5558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5735,6 +5874,18 @@
       <c r="B26" t="inlineStr">
         <is>
           <t>Monaco no Contadino, Spia, Capogilda; Fanatico della Guardia</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26-08-05_1</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Margherita vampirizzata</t>
         </is>
       </c>
     </row>
@@ -5750,7 +5901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6209,6 +6360,40 @@
       <c r="C27" t="inlineStr">
         <is>
           <t>Mago, Guardia, Azzeccagarbugli, Fanatico, Monaco, Veggente</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>26-08-05_1</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Villaggio, Giullare, Mistici</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Guaritore, Eremita, Giullare, Mercante, Veggente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>26-08-11_1</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Veggente, Contadino, Oratore, Medium, Mercante, Cacciatore di Vampiri</t>
         </is>
       </c>
     </row>
@@ -6224,7 +6409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6635,6 +6820,23 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>26-08-05_1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Margherita</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Vampiro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-08-11_2: Villaggio/Mistici/Giulietta/Romeo win (Traditore=Romeo). Fix 26-04-16_1: Pazzo (Margherita) did not actually win, remove from win/win_ruoli
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3009,7 +3009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AE38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3169,6 +3169,11 @@
           <t>26-08-11_1</t>
         </is>
       </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>26-08-11_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3301,6 +3306,11 @@
           <t>Medium</t>
         </is>
       </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3505,6 +3515,11 @@
           <t>Oratore</t>
         </is>
       </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3547,6 +3562,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>Altra Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4039,6 +4059,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4238,6 +4263,11 @@
           <t>Vampiro</t>
         </is>
       </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4512,6 +4542,11 @@
           <t>Mercante</t>
         </is>
       </c>
+      <c r="AE20" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4589,6 +4624,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AE21" t="inlineStr">
+        <is>
+          <t>Giulietta</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4805,6 +4845,11 @@
           <t>Cacciatore di Vampiri</t>
         </is>
       </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>Traditore</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4904,6 +4949,11 @@
           <t>Contadino</t>
         </is>
       </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4976,6 +5026,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5090,6 +5145,11 @@
           <t>Capobranco</t>
         </is>
       </c>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5142,6 +5202,11 @@
       <c r="Z36" t="inlineStr">
         <is>
           <t>Megera</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr">
+        <is>
+          <t>Oste</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5541,6 +5606,18 @@
         </is>
       </c>
       <c r="B29" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>26-08-11_2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
         </is>
@@ -5558,7 +5635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5886,6 +5963,18 @@
       <c r="B27" t="inlineStr">
         <is>
           <t>Margherita vampirizzata</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>26-08-11_2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Giulietta di Traditore</t>
         </is>
       </c>
     </row>
@@ -5901,7 +5990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6099,12 +6188,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Villaggio, Mistici, Pazzo, Angelo</t>
+          <t>Villaggio, Mistici, Angelo</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Prete, Bocca di Rosa, Mercante, Angelo, Pazzo, Medium, Guaritore, Veggente</t>
+          <t>Prete, Bocca di Rosa, Mercante, Angelo, Medium, Guaritore, Veggente</t>
         </is>
       </c>
     </row>
@@ -6394,6 +6483,23 @@
       <c r="C29" t="inlineStr">
         <is>
           <t>Veggente, Contadino, Oratore, Medium, Mercante, Cacciatore di Vampiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>26-08-11_2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici, Giulietta, Romeo</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Guardia, Oste, Eremita, Veggente, Medium, Traditore, Altra Guardia, Giulietta</t>
         </is>
       </c>
     </row>
@@ -6409,7 +6515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6837,6 +6943,23 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>26-08-11_2</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>TuBo97</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Romeo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add game 26-08-21_2: Capobranco (wolves) win. lippo=Andrea in this roster, giorgioc=Giorgio (not a new player)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3009,7 +3009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE38"/>
+  <dimension ref="A1:AF38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3174,6 +3174,11 @@
           <t>26-08-11_2</t>
         </is>
       </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>26-08-21_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3567,6 +3572,11 @@
           <t>Altra Guardia</t>
         </is>
       </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3706,6 +3716,11 @@
           <t>Bardo</t>
         </is>
       </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3803,6 +3818,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Oste</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -3957,6 +3977,11 @@
           <t>Assassino</t>
         </is>
       </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4064,6 +4089,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4268,6 +4298,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Traditore</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4365,6 +4400,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Oratore</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4419,6 +4459,11 @@
           <t>Azzeccagarbugli</t>
         </is>
       </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>Inquisitore</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4629,6 +4674,11 @@
           <t>Giulietta</t>
         </is>
       </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Giovane Lupo</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4954,6 +5004,11 @@
           <t>Eremita</t>
         </is>
       </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5031,6 +5086,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AF27" t="inlineStr">
+        <is>
+          <t>Guaritore</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5224,6 +5284,11 @@
       <c r="AB37" t="inlineStr">
         <is>
           <t>Giullare</t>
+        </is>
+      </c>
+      <c r="AF37" t="inlineStr">
+        <is>
+          <t>Monaco</t>
         </is>
       </c>
     </row>
@@ -5256,7 +5321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5620,6 +5685,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>26-08-21_2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Faida Inquisizione</t>
         </is>
       </c>
     </row>
@@ -5635,7 +5712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5975,6 +6052,18 @@
       <c r="B28" t="inlineStr">
         <is>
           <t>Giulietta di Traditore</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>26-08-21_2</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Monaco no Guardia, Altra Guardia, Vampiro</t>
         </is>
       </c>
     </row>
@@ -5990,7 +6079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6500,6 +6589,23 @@
       <c r="C30" t="inlineStr">
         <is>
           <t>Guardia, Oste, Eremita, Veggente, Medium, Traditore, Altra Guardia, Giulietta</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>26-08-21_2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Capobranco, Lupo del Branco, Traditore, Giovane Lupo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game 26-08-06_2: Villaggio/Angelo win (Amanti), Fanatico=Medium's Villaggio. Note: no 26-08-06_1 exists yet.
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3009,7 +3009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF38"/>
+  <dimension ref="A1:AG38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3179,6 +3179,11 @@
           <t>26-08-21_2</t>
         </is>
       </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>26-08-06_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3316,6 +3321,11 @@
           <t>Guardia</t>
         </is>
       </c>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3880,6 +3890,11 @@
           <t>Giullare</t>
         </is>
       </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -4094,6 +4109,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4303,6 +4323,11 @@
           <t>Traditore</t>
         </is>
       </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4405,6 +4430,11 @@
           <t>Oratore</t>
         </is>
       </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4592,6 +4622,11 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4900,6 +4935,11 @@
           <t>Traditore</t>
         </is>
       </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5306,6 +5346,11 @@
       <c r="AC38" t="inlineStr">
         <is>
           <t>Pazzo</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>Fanatico</t>
         </is>
       </c>
     </row>
@@ -5321,7 +5366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5697,6 +5742,18 @@
       <c r="B31" t="inlineStr">
         <is>
           <t>2 lune SÌ Faida Inquisizione</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>26-08-06_2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
         </is>
       </c>
     </row>
@@ -5712,7 +5769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6064,6 +6121,18 @@
       <c r="B29" t="inlineStr">
         <is>
           <t>Monaco no Guardia, Altra Guardia, Vampiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>26-08-06_2</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Fanatico del Medium; Angelo di Rosario</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6606,6 +6675,23 @@
       <c r="C31" t="inlineStr">
         <is>
           <t>Capobranco, Lupo del Branco, Traditore, Giovane Lupo</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>26-08-06_2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Villaggio, Angelo</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Medium, Fanatico, Angelo</t>
         </is>
       </c>
     </row>
@@ -6621,7 +6707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7066,6 +7152,23 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>26-08-06_2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Alessio</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Villaggio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rename 26-08-06_2 to 26-08-05_2 (was actually the second game of Aug 5)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3181,7 +3181,7 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
-          <t>26-08-06_2</t>
+          <t>26-08-05_2</t>
         </is>
       </c>
     </row>
@@ -5748,7 +5748,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>26-08-06_2</t>
+          <t>26-08-05_2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6127,7 +6127,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>26-08-06_2</t>
+          <t>26-08-05_2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6681,7 +6681,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>26-08-06_2</t>
+          <t>26-08-05_2</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -7155,7 +7155,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>26-08-06_2</t>
+          <t>26-08-05_2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">

</xml_diff>

<commit_message>
August games: Giullare means Giullare Modificato (Pietro 26-08-05_1, Andrea 26-08-21_1)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3887,7 +3887,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>Giullare</t>
+          <t>Giullare Modificato</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
@@ -5323,7 +5323,7 @@
       </c>
       <c r="AB37" t="inlineStr">
         <is>
-          <t>Giullare</t>
+          <t>Giullare Modificato</t>
         </is>
       </c>
       <c r="AF37" t="inlineStr">
@@ -6623,7 +6623,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Guaritore, Eremita, Giullare, Mercante, Veggente</t>
+          <t>Guaritore, Eremita, Giullare Modificato, Mercante, Veggente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix August games: 'lippo' was Andrea, not Filippo (26-08-11_1 Oratore, 26-08-11_2 Medium)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3525,16 +3525,6 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>Oratore</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5324,6 +5314,16 @@
       <c r="AB37" t="inlineStr">
         <is>
           <t>Giullare Modificato</t>
+        </is>
+      </c>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>Oratore</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="AF37" t="inlineStr">

</xml_diff>

<commit_message>
Add player Nulter (Marco); tag Andrea's nome with (Lippo); add game 26-08-27_1: Villaggio/Mistici win
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B38"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -904,7 +904,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Andrea</t>
+          <t>Andrea (Lippo)</t>
         </is>
       </c>
     </row>
@@ -917,6 +917,18 @@
       <c r="B38" t="inlineStr">
         <is>
           <t>Alessio</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Nulter</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Nulter (Marco)</t>
         </is>
       </c>
     </row>
@@ -3009,7 +3021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG38"/>
+  <dimension ref="A1:AH39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3184,6 +3196,11 @@
           <t>26-08-05_2</t>
         </is>
       </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>26-08-27_1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3525,6 +3542,11 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>Strega</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3619,6 +3641,11 @@
           <t>Mercante</t>
         </is>
       </c>
+      <c r="AH6" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4318,6 +4345,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>Altra Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4425,6 +4457,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AH14" t="inlineStr">
+        <is>
+          <t>Contadino</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4452,6 +4489,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AH15" t="inlineStr">
+        <is>
+          <t>Assassino</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4617,6 +4659,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="AH20" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4704,6 +4751,11 @@
           <t>Giovane Lupo</t>
         </is>
       </c>
+      <c r="AH21" t="inlineStr">
+        <is>
+          <t>Mercante</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5039,6 +5091,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5121,6 +5178,11 @@
           <t>Guaritore</t>
         </is>
       </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>Oste</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5331,6 +5393,11 @@
           <t>Monaco</t>
         </is>
       </c>
+      <c r="AH37" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5351,6 +5418,23 @@
       <c r="AG38" t="inlineStr">
         <is>
           <t>Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Nulter</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Nulter (Marco)</t>
+        </is>
+      </c>
+      <c r="AH39" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B32"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5754,6 +5838,18 @@
       <c r="B32" t="inlineStr">
         <is>
           <t>2 lune SÌ Capobranco Maledetto Fanatico</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>26-08-27_1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1 luna e 2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6692,6 +6788,23 @@
       <c r="C32" t="inlineStr">
         <is>
           <t>Medium, Fanatico, Angelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>26-08-27_1</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Villaggio, Mistici</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Medium, Veggente, Contadino, Mercante, Altra Guardia, Oste, Strega</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add players.alias column: alternate nicknames (e.g. Andrea's "Lippo") now show only in the Storico giocatore dropdown, not in nome (which stays clean everywhere else)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -475,6 +475,11 @@
           <t>Nome</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>alias</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -904,7 +909,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Andrea (Lippo)</t>
+          <t>Andrea</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Lippo</t>
         </is>
       </c>
     </row>
@@ -928,7 +938,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nulter (Marco)</t>
+          <t>Marco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add game 26-08-27_2: Capobranco win (Capobranco Maledetto, Lupo del Branco)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -3031,7 +3031,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH39"/>
+  <dimension ref="A1:AI39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="19.21875" customWidth="1" min="1" max="1"/>
@@ -3211,6 +3211,11 @@
           <t>26-08-27_1</t>
         </is>
       </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>26-08-27_2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3557,6 +3562,11 @@
           <t>Strega</t>
         </is>
       </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Oste</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3656,6 +3666,11 @@
           <t>Lupo del Branco</t>
         </is>
       </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4360,6 +4375,11 @@
           <t>Altra Guardia</t>
         </is>
       </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4472,6 +4492,11 @@
           <t>Contadino</t>
         </is>
       </c>
+      <c r="AI14" t="inlineStr">
+        <is>
+          <t>Veggente</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4504,6 +4529,11 @@
           <t>Assassino</t>
         </is>
       </c>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>Eremita</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4850,6 +4880,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>Prete</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5106,6 +5141,11 @@
           <t>Veggente</t>
         </is>
       </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>Guardia</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -5193,6 +5233,11 @@
           <t>Oste</t>
         </is>
       </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>Lupo del Branco</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5408,6 +5453,11 @@
           <t>Capobranco Maledetto</t>
         </is>
       </c>
+      <c r="AI37" t="inlineStr">
+        <is>
+          <t>Angelo</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -5445,6 +5495,11 @@
       <c r="AH39" t="inlineStr">
         <is>
           <t>Medium</t>
+        </is>
+      </c>
+      <c r="AI39" t="inlineStr">
+        <is>
+          <t>Assassino</t>
         </is>
       </c>
     </row>
@@ -5460,7 +5515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5858,6 +5913,18 @@
         </is>
       </c>
       <c r="B33" t="inlineStr">
+        <is>
+          <t>1 luna e 2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>26-08-27_2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>1 luna e 2 lune NO Giullare SÌ Capobranco Maledetto Fanatico Giullare Modificato</t>
         </is>
@@ -5875,7 +5942,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6239,6 +6306,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>Fanatico del Medium; Angelo di Rosario</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>26-08-27_2</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Prete custodito da Angelo</t>
         </is>
       </c>
     </row>
@@ -6254,7 +6333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.77734375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6815,6 +6894,23 @@
       <c r="C33" t="inlineStr">
         <is>
           <t>Medium, Veggente, Contadino, Mercante, Altra Guardia, Oste, Strega</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>26-08-27_2</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Capobranco</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Capobranco Maledetto, Lupo del Branco</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
26-08-27_2: add missing Master (Rosario)
</commit_message>
<xml_diff>
--- a/WWDiscordtemplate.xlsx
+++ b/WWDiscordtemplate.xlsx
@@ -4704,6 +4704,11 @@
           <t>MASTER</t>
         </is>
       </c>
+      <c r="AI20" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">

</xml_diff>